<commit_message>
Update QR codes with live domain https://kasbhunare-edu.vercel.app
</commit_message>
<xml_diff>
--- a/TALABALAR_QR_HAVOLALARI.xlsx
+++ b/TALABALAR_QR_HAVOLALARI.xlsx
@@ -489,7 +489,7 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>https://ilmziyo-cert.vercel.app/prof/pt/59aa66bf-01ac-4349-8870-5ff27af43771</t>
+          <t>https://kasbhunare-edu.vercel.app/prof/pt/59aa66bf-01ac-4349-8870-5ff27af43771</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
@@ -529,7 +529,7 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>https://ilmziyo-cert.vercel.app/prof/pt/cbeaf80d-81cb-4a84-99f8-c420550af4da</t>
+          <t>https://kasbhunare-edu.vercel.app/prof/pt/cbeaf80d-81cb-4a84-99f8-c420550af4da</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
@@ -569,7 +569,7 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>https://ilmziyo-cert.vercel.app/prof/pt/2214a045-60db-46a2-a6e2-95fe9dbc5998</t>
+          <t>https://kasbhunare-edu.vercel.app/prof/pt/2214a045-60db-46a2-a6e2-95fe9dbc5998</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
@@ -609,7 +609,7 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>https://ilmziyo-cert.vercel.app/prof/pt/22323ab1-a469-4948-aedd-f1e7a4c327d3</t>
+          <t>https://kasbhunare-edu.vercel.app/prof/pt/22323ab1-a469-4948-aedd-f1e7a4c327d3</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
@@ -649,7 +649,7 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>https://ilmziyo-cert.vercel.app/prof/pt/29b61334-e67c-4c3e-b5c3-0276cfaa9a3d</t>
+          <t>https://kasbhunare-edu.vercel.app/prof/pt/29b61334-e67c-4c3e-b5c3-0276cfaa9a3d</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -689,7 +689,7 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>https://ilmziyo-cert.vercel.app/prof/pt/43ab0e03-05a7-40f1-8b78-f79b8a178b06</t>
+          <t>https://kasbhunare-edu.vercel.app/prof/pt/43ab0e03-05a7-40f1-8b78-f79b8a178b06</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
@@ -729,7 +729,7 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>https://ilmziyo-cert.vercel.app/prof/pt/ecb73f90-927b-4f6f-8c1e-10637687b77f</t>
+          <t>https://kasbhunare-edu.vercel.app/prof/pt/ecb73f90-927b-4f6f-8c1e-10637687b77f</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
@@ -769,7 +769,7 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>https://ilmziyo-cert.vercel.app/prof/pt/2696b35e-e2ea-45cd-b6a1-c08dc2c21acc</t>
+          <t>https://kasbhunare-edu.vercel.app/prof/pt/2696b35e-e2ea-45cd-b6a1-c08dc2c21acc</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
@@ -809,7 +809,7 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>https://ilmziyo-cert.vercel.app/prof/pt/55fbbcec-826b-472f-9047-ebbf2c7c7318</t>
+          <t>https://kasbhunare-edu.vercel.app/prof/pt/55fbbcec-826b-472f-9047-ebbf2c7c7318</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
@@ -849,7 +849,7 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>https://ilmziyo-cert.vercel.app/prof/pt/3b568c98-fb63-41ea-9db1-e87bbaa8c214</t>
+          <t>https://kasbhunare-edu.vercel.app/prof/pt/3b568c98-fb63-41ea-9db1-e87bbaa8c214</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
@@ -889,7 +889,7 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>https://ilmziyo-cert.vercel.app/prof/pt/c408d39b-3773-4599-b1d0-0776f629eb0f</t>
+          <t>https://kasbhunare-edu.vercel.app/prof/pt/c408d39b-3773-4599-b1d0-0776f629eb0f</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
@@ -929,7 +929,7 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>https://ilmziyo-cert.vercel.app/prof/pt/a07b735a-c4f2-42c6-b479-74e01c905185</t>
+          <t>https://kasbhunare-edu.vercel.app/prof/pt/a07b735a-c4f2-42c6-b479-74e01c905185</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
@@ -969,7 +969,7 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>https://ilmziyo-cert.vercel.app/prof/pt/2c45c677-d7ee-4f77-9dae-ff936642c313</t>
+          <t>https://kasbhunare-edu.vercel.app/prof/pt/2c45c677-d7ee-4f77-9dae-ff936642c313</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
@@ -1009,7 +1009,7 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>https://ilmziyo-cert.vercel.app/prof/pt/eb11fac1-9b76-42e9-9d3b-709e33fdb34f</t>
+          <t>https://kasbhunare-edu.vercel.app/prof/pt/eb11fac1-9b76-42e9-9d3b-709e33fdb34f</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
@@ -1049,7 +1049,7 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>https://ilmziyo-cert.vercel.app/prof/pt/257fd4fc-1672-4e96-a568-8b592fe618ca</t>
+          <t>https://kasbhunare-edu.vercel.app/prof/pt/257fd4fc-1672-4e96-a568-8b592fe618ca</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
@@ -1089,7 +1089,7 @@
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>https://ilmziyo-cert.vercel.app/prof/pt/50746540-03bb-4794-b020-4a6b0366a7f9</t>
+          <t>https://kasbhunare-edu.vercel.app/prof/pt/50746540-03bb-4794-b020-4a6b0366a7f9</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
@@ -1129,7 +1129,7 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>https://ilmziyo-cert.vercel.app/prof/pt/19061955-7050-49e8-92ea-13d8810ef3bb</t>
+          <t>https://kasbhunare-edu.vercel.app/prof/pt/19061955-7050-49e8-92ea-13d8810ef3bb</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
@@ -1169,7 +1169,7 @@
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>https://ilmziyo-cert.vercel.app/prof/pt/3d60072c-72e1-4f52-9def-4bbdfee4f33b</t>
+          <t>https://kasbhunare-edu.vercel.app/prof/pt/3d60072c-72e1-4f52-9def-4bbdfee4f33b</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
@@ -1209,7 +1209,7 @@
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>https://ilmziyo-cert.vercel.app/prof/pt/fc30913b-14f1-4c0e-bfcf-fe839a35cd9b</t>
+          <t>https://kasbhunare-edu.vercel.app/prof/pt/fc30913b-14f1-4c0e-bfcf-fe839a35cd9b</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
@@ -1249,7 +1249,7 @@
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>https://ilmziyo-cert.vercel.app/prof/pt/d9b1040d-7b6d-4c54-af15-b8f68052ee96</t>
+          <t>https://kasbhunare-edu.vercel.app/prof/pt/d9b1040d-7b6d-4c54-af15-b8f68052ee96</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
@@ -1289,7 +1289,7 @@
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>https://ilmziyo-cert.vercel.app/prof/pt/86776295-fd6e-47bf-83e8-3af60466e709</t>
+          <t>https://kasbhunare-edu.vercel.app/prof/pt/86776295-fd6e-47bf-83e8-3af60466e709</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
@@ -1329,7 +1329,7 @@
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>https://ilmziyo-cert.vercel.app/prof/pt/f179e52e-633c-4873-bde9-c25b2aac26d0</t>
+          <t>https://kasbhunare-edu.vercel.app/prof/pt/f179e52e-633c-4873-bde9-c25b2aac26d0</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
@@ -1369,7 +1369,7 @@
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>https://ilmziyo-cert.vercel.app/prof/pt/20031802-d518-46a2-b254-f0b4ee4470c6</t>
+          <t>https://kasbhunare-edu.vercel.app/prof/pt/20031802-d518-46a2-b254-f0b4ee4470c6</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
@@ -1409,7 +1409,7 @@
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>https://ilmziyo-cert.vercel.app/prof/pt/357639c6-50cf-42a8-b43a-96c9c83160fc</t>
+          <t>https://kasbhunare-edu.vercel.app/prof/pt/357639c6-50cf-42a8-b43a-96c9c83160fc</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
@@ -1449,7 +1449,7 @@
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>https://ilmziyo-cert.vercel.app/prof/pt/44d8ca88-16d5-44a3-950d-f1e1f51d194c</t>
+          <t>https://kasbhunare-edu.vercel.app/prof/pt/44d8ca88-16d5-44a3-950d-f1e1f51d194c</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
@@ -1489,7 +1489,7 @@
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>https://ilmziyo-cert.vercel.app/prof/pt/e7eecd5c-3e69-4e33-bf9e-ef38aab320f5</t>
+          <t>https://kasbhunare-edu.vercel.app/prof/pt/e7eecd5c-3e69-4e33-bf9e-ef38aab320f5</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
@@ -1529,7 +1529,7 @@
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>https://ilmziyo-cert.vercel.app/prof/pt/a4ca945b-52d6-4fa5-965f-7eece002c917</t>
+          <t>https://kasbhunare-edu.vercel.app/prof/pt/a4ca945b-52d6-4fa5-965f-7eece002c917</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
@@ -1569,7 +1569,7 @@
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>https://ilmziyo-cert.vercel.app/prof/pt/fd7161a6-732a-4730-af50-bb529b2f4492</t>
+          <t>https://kasbhunare-edu.vercel.app/prof/pt/fd7161a6-732a-4730-af50-bb529b2f4492</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
@@ -1609,7 +1609,7 @@
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>https://ilmziyo-cert.vercel.app/prof/pt/448938fd-5c77-42ae-98be-77df54a8acee</t>
+          <t>https://kasbhunare-edu.vercel.app/prof/pt/448938fd-5c77-42ae-98be-77df54a8acee</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
@@ -1649,7 +1649,7 @@
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>https://ilmziyo-cert.vercel.app/prof/pt/4d508cae-d4ca-412d-82f9-27f5a15d91a7</t>
+          <t>https://kasbhunare-edu.vercel.app/prof/pt/4d508cae-d4ca-412d-82f9-27f5a15d91a7</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">

</xml_diff>

<commit_message>
Add high-res QR codes, styled Excel report and zip archive
</commit_message>
<xml_diff>
--- a/TALABALAR_QR_HAVOLALARI.xlsx
+++ b/TALABALAR_QR_HAVOLALARI.xlsx
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -25,13 +25,25 @@
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="11"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001F4E79"/>
+        <bgColor rgb="001F4E79"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -46,8 +58,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -413,46 +428,92 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H31"/>
+  <dimension ref="A1:N31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="37" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="17" customWidth="1" min="6" max="6"/>
+    <col width="28" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="40" customWidth="1" min="10" max="10"/>
+    <col width="13" customWidth="1" min="11" max="11"/>
+    <col width="13" customWidth="1" min="12" max="12"/>
+    <col width="81" customWidth="1" min="13" max="13"/>
+    <col width="39" customWidth="1" min="14" max="14"/>
+  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>T/R</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>F.I.O</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Sertifikat raqami</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Qayd raqami</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>JShShIR (PINFL)</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Tug'ilgan sana</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>Maxfiy QR Havola (Havolani o'zgartirib bo'lmaydi)</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Ta'lim muassasasi</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Mutaxassislik</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>O'quv soati</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>O'qish davri</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>DAK qarori</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>DAK sanasi</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>Jonli QR Havola</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>QR Fayl nomi</t>
         </is>
@@ -489,10 +550,40 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
+          <t>QARSHI TIBBIYOT TEXNIKUMI</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>Farmatsiya</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>360 soat</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>23.03.2026 yildan 13.06.2026 yilgacha</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>26/21</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>2026-06-13</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
           <t>https://kasbhunare-edu.vercel.app/prof/pt/59aa66bf-01ac-4349-8870-5ff27af43771</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr">
+      <c r="N2" t="inlineStr">
         <is>
           <t>01_ABDIXAKIMOVA_FAYOZA_0000001.png</t>
         </is>
@@ -529,10 +620,40 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
+          <t>QARSHI TIBBIYOT TEXNIKUMI</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>Farmatsiya</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>360 soat</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>23.03.2026 yildan 13.06.2026 yilgacha</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>26/21</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>2026-06-13</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
           <t>https://kasbhunare-edu.vercel.app/prof/pt/cbeaf80d-81cb-4a84-99f8-c420550af4da</t>
         </is>
       </c>
-      <c r="H3" t="inlineStr">
+      <c r="N3" t="inlineStr">
         <is>
           <t>02_ACHILOVA_NOZANIN_0000002.png</t>
         </is>
@@ -569,10 +690,40 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
+          <t>QARSHI TIBBIYOT TEXNIKUMI</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>Farmatsiya</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>360 soat</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>23.03.2026 yildan 13.06.2026 yilgacha</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>26/21</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>2026-06-13</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
           <t>https://kasbhunare-edu.vercel.app/prof/pt/2214a045-60db-46a2-a6e2-95fe9dbc5998</t>
         </is>
       </c>
-      <c r="H4" t="inlineStr">
+      <c r="N4" t="inlineStr">
         <is>
           <t>03_AXATOVA_INTIZOR_0000003.png</t>
         </is>
@@ -609,10 +760,40 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
+          <t>QARSHI TIBBIYOT TEXNIKUMI</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>Farmatsiya</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>360 soat</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>23.03.2026 yildan 13.06.2026 yilgacha</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>26/21</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>2026-06-13</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
           <t>https://kasbhunare-edu.vercel.app/prof/pt/22323ab1-a469-4948-aedd-f1e7a4c327d3</t>
         </is>
       </c>
-      <c r="H5" t="inlineStr">
+      <c r="N5" t="inlineStr">
         <is>
           <t>04_AXMADOVA_MUXLISA_0000004.png</t>
         </is>
@@ -649,10 +830,40 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
+          <t>QARSHI TIBBIYOT TEXNIKUMI</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>Farmatsiya</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>360 soat</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>23.03.2026 yildan 13.06.2026 yilgacha</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>26/21</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>2026-06-13</t>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
           <t>https://kasbhunare-edu.vercel.app/prof/pt/29b61334-e67c-4c3e-b5c3-0276cfaa9a3d</t>
         </is>
       </c>
-      <c r="H6" t="inlineStr">
+      <c r="N6" t="inlineStr">
         <is>
           <t>05_BOZOROVA_GULASAL_0000005.png</t>
         </is>
@@ -689,10 +900,40 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
+          <t>QARSHI TIBBIYOT TEXNIKUMI</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>Farmatsiya</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>360 soat</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>23.03.2026 yildan 13.06.2026 yilgacha</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>26/21</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>2026-06-13</t>
+        </is>
+      </c>
+      <c r="M7" t="inlineStr">
+        <is>
           <t>https://kasbhunare-edu.vercel.app/prof/pt/43ab0e03-05a7-40f1-8b78-f79b8a178b06</t>
         </is>
       </c>
-      <c r="H7" t="inlineStr">
+      <c r="N7" t="inlineStr">
         <is>
           <t>06_ESHMUXAMMADOVA_YULDUZ_0000006.png</t>
         </is>
@@ -729,10 +970,40 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
+          <t>QARSHI TIBBIYOT TEXNIKUMI</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>Farmatsiya</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>360 soat</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>23.03.2026 yildan 13.06.2026 yilgacha</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>26/21</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>2026-06-13</t>
+        </is>
+      </c>
+      <c r="M8" t="inlineStr">
+        <is>
           <t>https://kasbhunare-edu.vercel.app/prof/pt/ecb73f90-927b-4f6f-8c1e-10637687b77f</t>
         </is>
       </c>
-      <c r="H8" t="inlineStr">
+      <c r="N8" t="inlineStr">
         <is>
           <t>07_GAPPOROVA_MEHRINISO_0000007.png</t>
         </is>
@@ -769,10 +1040,40 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
+          <t>QARSHI TIBBIYOT TEXNIKUMI</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>Farmatsiya</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>360 soat</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>23.03.2026 yildan 13.06.2026 yilgacha</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>26/21</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>2026-06-13</t>
+        </is>
+      </c>
+      <c r="M9" t="inlineStr">
+        <is>
           <t>https://kasbhunare-edu.vercel.app/prof/pt/2696b35e-e2ea-45cd-b6a1-c08dc2c21acc</t>
         </is>
       </c>
-      <c r="H9" t="inlineStr">
+      <c r="N9" t="inlineStr">
         <is>
           <t>08_JAMOLOVA_OGILOY_0000008.png</t>
         </is>
@@ -809,10 +1110,40 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
+          <t>QARSHI TIBBIYOT TEXNIKUMI</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>Farmatsiya</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>360 soat</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>23.03.2026 yildan 13.06.2026 yilgacha</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>26/21</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>2026-06-13</t>
+        </is>
+      </c>
+      <c r="M10" t="inlineStr">
+        <is>
           <t>https://kasbhunare-edu.vercel.app/prof/pt/55fbbcec-826b-472f-9047-ebbf2c7c7318</t>
         </is>
       </c>
-      <c r="H10" t="inlineStr">
+      <c r="N10" t="inlineStr">
         <is>
           <t>09_JOVLIYEVA_RUHSHONA_0000009.png</t>
         </is>
@@ -849,10 +1180,40 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
+          <t>QARSHI TIBBIYOT TEXNIKUMI</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>Farmatsiya</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>360 soat</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>23.03.2026 yildan 13.06.2026 yilgacha</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>26/21</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>2026-06-13</t>
+        </is>
+      </c>
+      <c r="M11" t="inlineStr">
+        <is>
           <t>https://kasbhunare-edu.vercel.app/prof/pt/3b568c98-fb63-41ea-9db1-e87bbaa8c214</t>
         </is>
       </c>
-      <c r="H11" t="inlineStr">
+      <c r="N11" t="inlineStr">
         <is>
           <t>10_JURAQULOVA_ASLZODA_0000010.png</t>
         </is>
@@ -889,10 +1250,40 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
+          <t>QARSHI TIBBIYOT TEXNIKUMI</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>Farmatsiya</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>360 soat</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>23.03.2026 yildan 13.06.2026 yilgacha</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>26/21</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>2026-06-13</t>
+        </is>
+      </c>
+      <c r="M12" t="inlineStr">
+        <is>
           <t>https://kasbhunare-edu.vercel.app/prof/pt/c408d39b-3773-4599-b1d0-0776f629eb0f</t>
         </is>
       </c>
-      <c r="H12" t="inlineStr">
+      <c r="N12" t="inlineStr">
         <is>
           <t>11_KARIMOVA_RUXSHONA_0000011.png</t>
         </is>
@@ -929,10 +1320,40 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
+          <t>QARSHI TIBBIYOT TEXNIKUMI</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>Farmatsiya</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>360 soat</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>23.03.2026 yildan 13.06.2026 yilgacha</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>26/21</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>2026-06-13</t>
+        </is>
+      </c>
+      <c r="M13" t="inlineStr">
+        <is>
           <t>https://kasbhunare-edu.vercel.app/prof/pt/a07b735a-c4f2-42c6-b479-74e01c905185</t>
         </is>
       </c>
-      <c r="H13" t="inlineStr">
+      <c r="N13" t="inlineStr">
         <is>
           <t>12_MUSIRMONOVA_RUZIGUL_0000012.png</t>
         </is>
@@ -969,10 +1390,40 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
+          <t>QARSHI TIBBIYOT TEXNIKUMI</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>Farmatsiya</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>360 soat</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>23.03.2026 yildan 13.06.2026 yilgacha</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>26/21</t>
+        </is>
+      </c>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>2026-06-13</t>
+        </is>
+      </c>
+      <c r="M14" t="inlineStr">
+        <is>
           <t>https://kasbhunare-edu.vercel.app/prof/pt/2c45c677-d7ee-4f77-9dae-ff936642c313</t>
         </is>
       </c>
-      <c r="H14" t="inlineStr">
+      <c r="N14" t="inlineStr">
         <is>
           <t>13_NASRULLAYEVA_BAHORA_0000013.png</t>
         </is>
@@ -1009,10 +1460,40 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
+          <t>QARSHI TIBBIYOT TEXNIKUMI</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>Farmatsiya</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>360 soat</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>23.03.2026 yildan 13.06.2026 yilgacha</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>26/21</t>
+        </is>
+      </c>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t>2026-06-13</t>
+        </is>
+      </c>
+      <c r="M15" t="inlineStr">
+        <is>
           <t>https://kasbhunare-edu.vercel.app/prof/pt/eb11fac1-9b76-42e9-9d3b-709e33fdb34f</t>
         </is>
       </c>
-      <c r="H15" t="inlineStr">
+      <c r="N15" t="inlineStr">
         <is>
           <t>14_NORMAMATOVA_SHAYDO_0000014.png</t>
         </is>
@@ -1049,10 +1530,40 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
+          <t>QARSHI TIBBIYOT TEXNIKUMI</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>Farmatsiya</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>360 soat</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>23.03.2026 yildan 13.06.2026 yilgacha</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>26/21</t>
+        </is>
+      </c>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>2026-06-13</t>
+        </is>
+      </c>
+      <c r="M16" t="inlineStr">
+        <is>
           <t>https://kasbhunare-edu.vercel.app/prof/pt/257fd4fc-1672-4e96-a568-8b592fe618ca</t>
         </is>
       </c>
-      <c r="H16" t="inlineStr">
+      <c r="N16" t="inlineStr">
         <is>
           <t>15_NORMURODOVA_MARJONA_0000015.png</t>
         </is>
@@ -1089,10 +1600,40 @@
       </c>
       <c r="G17" t="inlineStr">
         <is>
+          <t>QARSHI TIBBIYOT TEXNIKUMI</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>Farmatsiya</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>360 soat</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>23.03.2026 yildan 13.06.2026 yilgacha</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>26/21</t>
+        </is>
+      </c>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>2026-06-13</t>
+        </is>
+      </c>
+      <c r="M17" t="inlineStr">
+        <is>
           <t>https://kasbhunare-edu.vercel.app/prof/pt/50746540-03bb-4794-b020-4a6b0366a7f9</t>
         </is>
       </c>
-      <c r="H17" t="inlineStr">
+      <c r="N17" t="inlineStr">
         <is>
           <t>16_ORIFOVA_SHAXLO_0000016.png</t>
         </is>
@@ -1129,10 +1670,40 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
+          <t>QARSHI TIBBIYOT TEXNIKUMI</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>Farmatsiya</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>360 soat</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>23.03.2026 yildan 13.06.2026 yilgacha</t>
+        </is>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>26/21</t>
+        </is>
+      </c>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t>2026-06-13</t>
+        </is>
+      </c>
+      <c r="M18" t="inlineStr">
+        <is>
           <t>https://kasbhunare-edu.vercel.app/prof/pt/19061955-7050-49e8-92ea-13d8810ef3bb</t>
         </is>
       </c>
-      <c r="H18" t="inlineStr">
+      <c r="N18" t="inlineStr">
         <is>
           <t>17_OROQOVA_RAYHONA_0000017.png</t>
         </is>
@@ -1169,10 +1740,40 @@
       </c>
       <c r="G19" t="inlineStr">
         <is>
+          <t>QARSHI TIBBIYOT TEXNIKUMI</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>Farmatsiya</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>360 soat</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>23.03.2026 yildan 13.06.2026 yilgacha</t>
+        </is>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>26/21</t>
+        </is>
+      </c>
+      <c r="L19" t="inlineStr">
+        <is>
+          <t>2026-06-13</t>
+        </is>
+      </c>
+      <c r="M19" t="inlineStr">
+        <is>
           <t>https://kasbhunare-edu.vercel.app/prof/pt/3d60072c-72e1-4f52-9def-4bbdfee4f33b</t>
         </is>
       </c>
-      <c r="H19" t="inlineStr">
+      <c r="N19" t="inlineStr">
         <is>
           <t>18_PULATOVA_SUMBULA_0000018.png</t>
         </is>
@@ -1209,10 +1810,40 @@
       </c>
       <c r="G20" t="inlineStr">
         <is>
+          <t>QARSHI TIBBIYOT TEXNIKUMI</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>Farmatsiya</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>360 soat</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>23.03.2026 yildan 13.06.2026 yilgacha</t>
+        </is>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>26/21</t>
+        </is>
+      </c>
+      <c r="L20" t="inlineStr">
+        <is>
+          <t>2026-06-13</t>
+        </is>
+      </c>
+      <c r="M20" t="inlineStr">
+        <is>
           <t>https://kasbhunare-edu.vercel.app/prof/pt/fc30913b-14f1-4c0e-bfcf-fe839a35cd9b</t>
         </is>
       </c>
-      <c r="H20" t="inlineStr">
+      <c r="N20" t="inlineStr">
         <is>
           <t>19_RAHMONOVA_LAZIZA_0000019.png</t>
         </is>
@@ -1249,10 +1880,40 @@
       </c>
       <c r="G21" t="inlineStr">
         <is>
+          <t>QARSHI TIBBIYOT TEXNIKUMI</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>Farmatsiya</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>360 soat</t>
+        </is>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>23.03.2026 yildan 13.06.2026 yilgacha</t>
+        </is>
+      </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>26/21</t>
+        </is>
+      </c>
+      <c r="L21" t="inlineStr">
+        <is>
+          <t>2026-06-13</t>
+        </is>
+      </c>
+      <c r="M21" t="inlineStr">
+        <is>
           <t>https://kasbhunare-edu.vercel.app/prof/pt/d9b1040d-7b6d-4c54-af15-b8f68052ee96</t>
         </is>
       </c>
-      <c r="H21" t="inlineStr">
+      <c r="N21" t="inlineStr">
         <is>
           <t>20_RAUPOVA_DILRABO_0000020.png</t>
         </is>
@@ -1289,10 +1950,40 @@
       </c>
       <c r="G22" t="inlineStr">
         <is>
+          <t>QARSHI TIBBIYOT TEXNIKUMI</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>Farmatsiya</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>360 soat</t>
+        </is>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>23.03.2026 yildan 13.06.2026 yilgacha</t>
+        </is>
+      </c>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>26/21</t>
+        </is>
+      </c>
+      <c r="L22" t="inlineStr">
+        <is>
+          <t>2026-06-13</t>
+        </is>
+      </c>
+      <c r="M22" t="inlineStr">
+        <is>
           <t>https://kasbhunare-edu.vercel.app/prof/pt/86776295-fd6e-47bf-83e8-3af60466e709</t>
         </is>
       </c>
-      <c r="H22" t="inlineStr">
+      <c r="N22" t="inlineStr">
         <is>
           <t>21_RUSTAMOVA_UGILOY_0000021.png</t>
         </is>
@@ -1329,10 +2020,40 @@
       </c>
       <c r="G23" t="inlineStr">
         <is>
+          <t>QARSHI TIBBIYOT TEXNIKUMI</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>Farmatsiya</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>360 soat</t>
+        </is>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>23.03.2026 yildan 13.06.2026 yilgacha</t>
+        </is>
+      </c>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>26/21</t>
+        </is>
+      </c>
+      <c r="L23" t="inlineStr">
+        <is>
+          <t>2026-06-13</t>
+        </is>
+      </c>
+      <c r="M23" t="inlineStr">
+        <is>
           <t>https://kasbhunare-edu.vercel.app/prof/pt/f179e52e-633c-4873-bde9-c25b2aac26d0</t>
         </is>
       </c>
-      <c r="H23" t="inlineStr">
+      <c r="N23" t="inlineStr">
         <is>
           <t>22_SAYFULLAYEVA_GULLOLA_0000022.png</t>
         </is>
@@ -1369,10 +2090,40 @@
       </c>
       <c r="G24" t="inlineStr">
         <is>
+          <t>QARSHI TIBBIYOT TEXNIKUMI</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>Farmatsiya</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>360 soat</t>
+        </is>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>23.03.2026 yildan 13.06.2026 yilgacha</t>
+        </is>
+      </c>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>26/21</t>
+        </is>
+      </c>
+      <c r="L24" t="inlineStr">
+        <is>
+          <t>2026-06-13</t>
+        </is>
+      </c>
+      <c r="M24" t="inlineStr">
+        <is>
           <t>https://kasbhunare-edu.vercel.app/prof/pt/20031802-d518-46a2-b254-f0b4ee4470c6</t>
         </is>
       </c>
-      <c r="H24" t="inlineStr">
+      <c r="N24" t="inlineStr">
         <is>
           <t>23_SUYAROVA_MALIKA_0000023.png</t>
         </is>
@@ -1409,10 +2160,40 @@
       </c>
       <c r="G25" t="inlineStr">
         <is>
+          <t>QARSHI TIBBIYOT TEXNIKUMI</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>Farmatsiya</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>360 soat</t>
+        </is>
+      </c>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>23.03.2026 yildan 13.06.2026 yilgacha</t>
+        </is>
+      </c>
+      <c r="K25" t="inlineStr">
+        <is>
+          <t>26/21</t>
+        </is>
+      </c>
+      <c r="L25" t="inlineStr">
+        <is>
+          <t>2026-06-13</t>
+        </is>
+      </c>
+      <c r="M25" t="inlineStr">
+        <is>
           <t>https://kasbhunare-edu.vercel.app/prof/pt/357639c6-50cf-42a8-b43a-96c9c83160fc</t>
         </is>
       </c>
-      <c r="H25" t="inlineStr">
+      <c r="N25" t="inlineStr">
         <is>
           <t>24_TURSUNOVA_AZIZA_0000024.png</t>
         </is>
@@ -1449,10 +2230,40 @@
       </c>
       <c r="G26" t="inlineStr">
         <is>
+          <t>QARSHI TIBBIYOT TEXNIKUMI</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>Farmatsiya</t>
+        </is>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>360 soat</t>
+        </is>
+      </c>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>23.03.2026 yildan 13.06.2026 yilgacha</t>
+        </is>
+      </c>
+      <c r="K26" t="inlineStr">
+        <is>
+          <t>26/21</t>
+        </is>
+      </c>
+      <c r="L26" t="inlineStr">
+        <is>
+          <t>2026-06-13</t>
+        </is>
+      </c>
+      <c r="M26" t="inlineStr">
+        <is>
           <t>https://kasbhunare-edu.vercel.app/prof/pt/44d8ca88-16d5-44a3-950d-f1e1f51d194c</t>
         </is>
       </c>
-      <c r="H26" t="inlineStr">
+      <c r="N26" t="inlineStr">
         <is>
           <t>25_TUYCHIYEVA_SEVARA_0000025.png</t>
         </is>
@@ -1489,10 +2300,40 @@
       </c>
       <c r="G27" t="inlineStr">
         <is>
+          <t>QARSHI TIBBIYOT TEXNIKUMI</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>Farmatsiya</t>
+        </is>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>360 soat</t>
+        </is>
+      </c>
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>23.03.2026 yildan 13.06.2026 yilgacha</t>
+        </is>
+      </c>
+      <c r="K27" t="inlineStr">
+        <is>
+          <t>26/21</t>
+        </is>
+      </c>
+      <c r="L27" t="inlineStr">
+        <is>
+          <t>2026-06-13</t>
+        </is>
+      </c>
+      <c r="M27" t="inlineStr">
+        <is>
           <t>https://kasbhunare-edu.vercel.app/prof/pt/e7eecd5c-3e69-4e33-bf9e-ef38aab320f5</t>
         </is>
       </c>
-      <c r="H27" t="inlineStr">
+      <c r="N27" t="inlineStr">
         <is>
           <t>26_XALILOVA_GOZAL_0000026.png</t>
         </is>
@@ -1529,10 +2370,40 @@
       </c>
       <c r="G28" t="inlineStr">
         <is>
+          <t>QARSHI TIBBIYOT TEXNIKUMI</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>Farmatsiya</t>
+        </is>
+      </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>360 soat</t>
+        </is>
+      </c>
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>23.03.2026 yildan 13.06.2026 yilgacha</t>
+        </is>
+      </c>
+      <c r="K28" t="inlineStr">
+        <is>
+          <t>26/21</t>
+        </is>
+      </c>
+      <c r="L28" t="inlineStr">
+        <is>
+          <t>2026-06-13</t>
+        </is>
+      </c>
+      <c r="M28" t="inlineStr">
+        <is>
           <t>https://kasbhunare-edu.vercel.app/prof/pt/a4ca945b-52d6-4fa5-965f-7eece002c917</t>
         </is>
       </c>
-      <c r="H28" t="inlineStr">
+      <c r="N28" t="inlineStr">
         <is>
           <t>27_XALIMOVA_SEVELA_0000027.png</t>
         </is>
@@ -1569,10 +2440,40 @@
       </c>
       <c r="G29" t="inlineStr">
         <is>
+          <t>QARSHI TIBBIYOT TEXNIKUMI</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>Farmatsiya</t>
+        </is>
+      </c>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>360 soat</t>
+        </is>
+      </c>
+      <c r="J29" t="inlineStr">
+        <is>
+          <t>23.03.2026 yildan 13.06.2026 yilgacha</t>
+        </is>
+      </c>
+      <c r="K29" t="inlineStr">
+        <is>
+          <t>26/21</t>
+        </is>
+      </c>
+      <c r="L29" t="inlineStr">
+        <is>
+          <t>2026-06-13</t>
+        </is>
+      </c>
+      <c r="M29" t="inlineStr">
+        <is>
           <t>https://kasbhunare-edu.vercel.app/prof/pt/fd7161a6-732a-4730-af50-bb529b2f4492</t>
         </is>
       </c>
-      <c r="H29" t="inlineStr">
+      <c r="N29" t="inlineStr">
         <is>
           <t>28_XURRAMOVA_ZARIFA_0000028.png</t>
         </is>
@@ -1609,10 +2510,40 @@
       </c>
       <c r="G30" t="inlineStr">
         <is>
+          <t>QARSHI TIBBIYOT TEXNIKUMI</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>Farmatsiya</t>
+        </is>
+      </c>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>360 soat</t>
+        </is>
+      </c>
+      <c r="J30" t="inlineStr">
+        <is>
+          <t>23.03.2026 yildan 13.06.2026 yilgacha</t>
+        </is>
+      </c>
+      <c r="K30" t="inlineStr">
+        <is>
+          <t>26/21</t>
+        </is>
+      </c>
+      <c r="L30" t="inlineStr">
+        <is>
+          <t>2026-06-13</t>
+        </is>
+      </c>
+      <c r="M30" t="inlineStr">
+        <is>
           <t>https://kasbhunare-edu.vercel.app/prof/pt/448938fd-5c77-42ae-98be-77df54a8acee</t>
         </is>
       </c>
-      <c r="H30" t="inlineStr">
+      <c r="N30" t="inlineStr">
         <is>
           <t>29_YUSUPOVA_DILSHODA_0000029.png</t>
         </is>
@@ -1649,10 +2580,40 @@
       </c>
       <c r="G31" t="inlineStr">
         <is>
+          <t>QARSHI TIBBIYOT TEXNIKUMI</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>Farmatsiya</t>
+        </is>
+      </c>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>360 soat</t>
+        </is>
+      </c>
+      <c r="J31" t="inlineStr">
+        <is>
+          <t>23.03.2026 yildan 13.06.2026 yilgacha</t>
+        </is>
+      </c>
+      <c r="K31" t="inlineStr">
+        <is>
+          <t>26/21</t>
+        </is>
+      </c>
+      <c r="L31" t="inlineStr">
+        <is>
+          <t>2026-06-13</t>
+        </is>
+      </c>
+      <c r="M31" t="inlineStr">
+        <is>
           <t>https://kasbhunare-edu.vercel.app/prof/pt/4d508cae-d4ca-412d-82f9-27f5a15d91a7</t>
         </is>
       </c>
-      <c r="H31" t="inlineStr">
+      <c r="N31" t="inlineStr">
         <is>
           <t>30_ZIYOVIDDINOVA_LAYLO_0000030.png</t>
         </is>

</xml_diff>

<commit_message>
Update DAK sanasi to 2026-06-15
</commit_message>
<xml_diff>
--- a/TALABALAR_QR_HAVOLALARI.xlsx
+++ b/TALABALAR_QR_HAVOLALARI.xlsx
@@ -575,7 +575,7 @@
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
@@ -645,7 +645,7 @@
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
@@ -715,7 +715,7 @@
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
@@ -785,7 +785,7 @@
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
@@ -855,7 +855,7 @@
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
@@ -925,7 +925,7 @@
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
@@ -995,7 +995,7 @@
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
@@ -1065,7 +1065,7 @@
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
@@ -1135,7 +1135,7 @@
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="M10" t="inlineStr">
@@ -1205,7 +1205,7 @@
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="M11" t="inlineStr">
@@ -1275,7 +1275,7 @@
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="M12" t="inlineStr">
@@ -1345,7 +1345,7 @@
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="M13" t="inlineStr">
@@ -1415,7 +1415,7 @@
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="M14" t="inlineStr">
@@ -1485,7 +1485,7 @@
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
@@ -1555,7 +1555,7 @@
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="M16" t="inlineStr">
@@ -1625,7 +1625,7 @@
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="M17" t="inlineStr">
@@ -1695,7 +1695,7 @@
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="M18" t="inlineStr">
@@ -1765,7 +1765,7 @@
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="M19" t="inlineStr">
@@ -1835,7 +1835,7 @@
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="M20" t="inlineStr">
@@ -1905,7 +1905,7 @@
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="M21" t="inlineStr">
@@ -1975,7 +1975,7 @@
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="M22" t="inlineStr">
@@ -2045,7 +2045,7 @@
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="M23" t="inlineStr">
@@ -2115,7 +2115,7 @@
       </c>
       <c r="L24" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="M24" t="inlineStr">
@@ -2185,7 +2185,7 @@
       </c>
       <c r="L25" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="M25" t="inlineStr">
@@ -2255,7 +2255,7 @@
       </c>
       <c r="L26" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="M26" t="inlineStr">
@@ -2325,7 +2325,7 @@
       </c>
       <c r="L27" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="M27" t="inlineStr">
@@ -2395,7 +2395,7 @@
       </c>
       <c r="L28" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="M28" t="inlineStr">
@@ -2465,7 +2465,7 @@
       </c>
       <c r="L29" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="M29" t="inlineStr">
@@ -2535,7 +2535,7 @@
       </c>
       <c r="L30" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="M30" t="inlineStr">
@@ -2605,7 +2605,7 @@
       </c>
       <c r="L31" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="M31" t="inlineStr">

</xml_diff>

<commit_message>
Add student 31 Tursunova Mohinur (Logopediya) and generate QR code
</commit_message>
<xml_diff>
--- a/TALABALAR_QR_HAVOLALARI.xlsx
+++ b/TALABALAR_QR_HAVOLALARI.xlsx
@@ -428,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N31"/>
+  <dimension ref="A1:N32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2619,6 +2619,76 @@
         </is>
       </c>
     </row>
+    <row r="32">
+      <c r="A32" t="n">
+        <v>31</v>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>TURSUNOVA MOHINUR JO'RABEK QIZI</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>QT L&amp;P № 0000031</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>0000031</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>61607025680034</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>2002-07-16</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>QARSHI TIBBIYOT TEXNIKUMI</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>Logopediya</t>
+        </is>
+      </c>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>360 soat</t>
+        </is>
+      </c>
+      <c r="J32" t="inlineStr">
+        <is>
+          <t>23.03.2026 yildan 13.06.2026 yilgacha</t>
+        </is>
+      </c>
+      <c r="K32" t="inlineStr">
+        <is>
+          <t>26/21</t>
+        </is>
+      </c>
+      <c r="L32" t="inlineStr">
+        <is>
+          <t>2026-06-15</t>
+        </is>
+      </c>
+      <c r="M32" t="inlineStr">
+        <is>
+          <t>https://kasbhunare-edu.vercel.app/prof/pt/e60fbcb2-ee31-432c-bdd5-326f5624fa76</t>
+        </is>
+      </c>
+      <c r="N32" t="inlineStr">
+        <is>
+          <t>31_TURSUNOVA_MOHINUR_0000031.png</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>